<commit_message>
feat: add clip preview, management, and cross-platform posting functionality for v2 dashboard
</commit_message>
<xml_diff>
--- a/AI Api Pricing/Gemini_API_Pricing_Summary_2026.xlsx
+++ b/AI Api Pricing/Gemini_API_Pricing_Summary_2026.xlsx
@@ -12,15 +12,19 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12480"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview &amp; Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="API Pricing Reference" sheetId="2" r:id="rId2"/>
+    <sheet name="Cost Finder" sheetId="3" r:id="rId1"/>
+    <sheet name="Overview &amp; Summary" sheetId="1" r:id="rId2"/>
+    <sheet name="API Pricing Reference" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cost Finder'!$A$1:$E$36</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="131">
   <si>
     <t>Google Gemini Developer API Pricing Summary</t>
   </si>
@@ -254,19 +258,180 @@
   </si>
   <si>
     <t>IN PKR</t>
+  </si>
+  <si>
+    <t>Provider</t>
+  </si>
+  <si>
+    <t>Service Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Pricing</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>ECS</t>
+  </si>
+  <si>
+    <t>Lambda</t>
+  </si>
+  <si>
+    <t>Service</t>
+  </si>
+  <si>
+    <t>Face Tracking</t>
+  </si>
+  <si>
+    <t>Video Rendering</t>
+  </si>
+  <si>
+    <t>Pricing Unit</t>
+  </si>
+  <si>
+    <t>Elevenlabs</t>
+  </si>
+  <si>
+    <t>Scribe v1 / v2</t>
+  </si>
+  <si>
+    <t>Speech to Text</t>
+  </si>
+  <si>
+    <t>per hour</t>
+  </si>
+  <si>
+    <t>per 1 min render</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>Video Analysis</t>
+  </si>
+  <si>
+    <t>per 20 min video</t>
+  </si>
+  <si>
+    <t>Supabase</t>
+  </si>
+  <si>
+    <t>Pro Subscription</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>per month (Flat)</t>
+  </si>
+  <si>
+    <t>Vercel</t>
+  </si>
+  <si>
+    <t>Website Hosting</t>
+  </si>
+  <si>
+    <t>Hostinger</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>per year (Flat)</t>
+  </si>
+  <si>
+    <t>Other Charges &amp; Fees</t>
+  </si>
+  <si>
+    <t>SECP Incorporation</t>
+  </si>
+  <si>
+    <t>Registration Step</t>
+  </si>
+  <si>
+    <t>Estimated Cost (PKR)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Combined fee for name reservation and digital SMC registration via the LEAP portal.</t>
+  </si>
+  <si>
+    <t>IT Startup tier (for businesses operating for less than 12 months).</t>
+  </si>
+  <si>
+    <t>Only applicable if you hire a tax lawyer/agency to handle the filings for you.</t>
+  </si>
+  <si>
+    <t>PSEB Registration</t>
+  </si>
+  <si>
+    <t>Consultant Fees (Optional)</t>
+  </si>
+  <si>
+    <t>Total Estimated Budget</t>
+  </si>
+  <si>
+    <t>Paddle</t>
+  </si>
+  <si>
+    <t>Payment Gateway</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>5% + $0.50</t>
+  </si>
+  <si>
+    <t>per Checkout transaction</t>
+  </si>
+  <si>
+    <t>Twenty2Short Cost Estimate</t>
+  </si>
+  <si>
+    <t>Services Description:</t>
+  </si>
+  <si>
+    <t>Estimated cost per 20 min video by service:</t>
+  </si>
+  <si>
+    <t>Cost per video</t>
+  </si>
+  <si>
+    <t>Net Cost Per Video</t>
+  </si>
+  <si>
+    <t>per GB per month</t>
+  </si>
+  <si>
+    <t>Vidoe Duration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="170" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0.000_ ;_-[$$-409]* \-#,##0.000\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="177" formatCode="General&quot;min&quot;"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,36 +444,65 @@
       <sz val="16"/>
       <color rgb="FF1B365D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF555555"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color rgb="FF1B365D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -341,7 +535,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -364,12 +558,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -402,8 +644,79 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -707,6 +1020,416 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:E36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.5703125" style="20" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" style="21" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" style="22" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5"/>
+      <c r="E5"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="41"/>
+      <c r="C6" s="28"/>
+      <c r="D6"/>
+      <c r="E6"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="41"/>
+      <c r="C7" s="28"/>
+      <c r="D7"/>
+      <c r="E7"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="43" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="41"/>
+      <c r="C8" s="28"/>
+      <c r="D8"/>
+      <c r="E8"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="43" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="41"/>
+      <c r="C9" s="28"/>
+      <c r="D9"/>
+      <c r="E9"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="41"/>
+      <c r="C10" s="28"/>
+      <c r="D10"/>
+      <c r="E10"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="41"/>
+      <c r="C11" s="28"/>
+      <c r="D11"/>
+      <c r="E11"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="41"/>
+      <c r="C12" s="28"/>
+      <c r="D12"/>
+      <c r="E12"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="43" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" s="41"/>
+      <c r="C13" s="28"/>
+      <c r="D13"/>
+      <c r="E13"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="41"/>
+      <c r="C14" s="28"/>
+      <c r="D14"/>
+      <c r="E14"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="39"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20" s="27">
+        <v>2.3E-2</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="27">
+        <v>0.04</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" s="27">
+        <v>0.01</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="27">
+        <v>0.22</v>
+      </c>
+      <c r="E23" s="28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="27">
+        <v>0.1</v>
+      </c>
+      <c r="E24" s="28" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="D25" s="27">
+        <v>25</v>
+      </c>
+      <c r="E25" s="28" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D26" s="27">
+        <v>20</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="27">
+        <v>15</v>
+      </c>
+      <c r="E27" s="28" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="E28" s="28" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="35"/>
+      <c r="C31" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="E31" s="35"/>
+    </row>
+    <row r="32" spans="1:5" s="30" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="34">
+        <v>10625</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="E32" s="36"/>
+    </row>
+    <row r="33" spans="1:5" s="30" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="B33" s="33"/>
+      <c r="C33" s="34">
+        <v>5000</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="E33" s="36"/>
+    </row>
+    <row r="34" spans="1:5" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" s="33"/>
+      <c r="C34" s="34">
+        <v>20000</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="E34" s="36"/>
+    </row>
+    <row r="35" spans="1:5" s="30" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B35" s="37"/>
+      <c r="C35" s="38">
+        <f>SUM(C32:C34)</f>
+        <v>35625</v>
+      </c>
+      <c r="D35" s="31"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -777,15 +1500,15 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
     </row>
     <row r="13" spans="1:11" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
@@ -987,12 +1710,12 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
@@ -1083,12 +1806,12 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A33" s="18" t="s">
+      <c r="A33" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
@@ -1188,7 +1911,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1604,7 +2327,7 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E29" s="19">
+      <c r="E29" s="18">
         <v>6.0002400096003798E-5</v>
       </c>
     </row>

</xml_diff>